<commit_message>
name the module rows from their own ora, the kept list had drifted off the network
</commit_message>
<xml_diff>
--- a/04_Figures/F04_association/modules/c_data/F04_modules_source_data.xlsx
+++ b/04_Figures/F04_association/modules/c_data/F04_modules_source_data.xlsx
@@ -133,7 +133,7 @@
     <t xml:space="preserve">no enriched term</t>
   </si>
   <si>
-    <t xml:space="preserve">Turquoise</t>
+    <t xml:space="preserve">Turquoise - no enriched term</t>
   </si>
   <si>
     <t xml:space="preserve">blue</t>
@@ -143,7 +143,7 @@
 metabolic process</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue - RNA Splicing*</t>
+    <t xml:space="preserve">Blue - small molecule metabolic pr...</t>
   </si>
   <si>
     <t xml:space="preserve">brown</t>
@@ -153,7 +153,7 @@
 organization</t>
   </si>
   <si>
-    <t xml:space="preserve">Brown - Amino Acid Metabolism</t>
+    <t xml:space="preserve">Brown - cytoskeleton organization</t>
   </si>
   <si>
     <t xml:space="preserve">yellow</t>
@@ -164,25 +164,25 @@
 organic...</t>
   </si>
   <si>
-    <t xml:space="preserve">Yellow - Small-Molecule Metabolism</t>
+    <t xml:space="preserve">Yellow - energy derivation by oxidat...</t>
   </si>
   <si>
     <t xml:space="preserve">green</t>
   </si>
   <si>
-    <t xml:space="preserve">Green</t>
+    <t xml:space="preserve">Green - no enriched term</t>
   </si>
   <si>
     <t xml:space="preserve">red</t>
   </si>
   <si>
-    <t xml:space="preserve">Red</t>
+    <t xml:space="preserve">Red - no enriched term</t>
   </si>
   <si>
     <t xml:space="preserve">black</t>
   </si>
   <si>
-    <t xml:space="preserve">Black - Aerobic Respiration</t>
+    <t xml:space="preserve">Black - no enriched term</t>
   </si>
   <si>
     <t xml:space="preserve">pink</t>
@@ -192,7 +192,7 @@
 process</t>
   </si>
   <si>
-    <t xml:space="preserve">Pink - Cytoplasmic Translation</t>
+    <t xml:space="preserve">Pink - actin filament-based process</t>
   </si>
   <si>
     <t xml:space="preserve">magenta</t>
@@ -202,13 +202,13 @@
 translation</t>
   </si>
   <si>
-    <t xml:space="preserve">Magenta - Sarcomere / Myofibril</t>
+    <t xml:space="preserve">Magenta - cytoplasmic translation</t>
   </si>
   <si>
     <t xml:space="preserve">purple</t>
   </si>
   <si>
-    <t xml:space="preserve">Purple - Translation (secondary)</t>
+    <t xml:space="preserve">Purple - cytoplasmic translation</t>
   </si>
   <si>
     <t xml:space="preserve">greenyellow</t>
@@ -218,7 +218,7 @@
 organization</t>
   </si>
   <si>
-    <t xml:space="preserve">Greenyellow - Electron Transport Chain</t>
+    <t xml:space="preserve">Greenyellow - extracellular matrix organi...</t>
   </si>
   <si>
     <t xml:space="preserve">tan</t>
@@ -228,7 +228,7 @@
 transport chain</t>
   </si>
   <si>
-    <t xml:space="preserve">Tan</t>
+    <t xml:space="preserve">Tan - aerobic electron transport ...</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
drop fry from pathway testing, singscore and fgsea only as agreed
</commit_message>
<xml_diff>
--- a/04_Figures/F04_association/modules/c_data/F04_modules_source_data.xlsx
+++ b/04_Figures/F04_association/modules/c_data/F04_modules_source_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t xml:space="preserve">feature</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t xml:space="preserve">n_annotated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fry_fdr</t>
   </si>
   <si>
     <t xml:space="preserve">ME_black</t>
@@ -582,19 +579,16 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>0.106679111156521</v>
@@ -607,17 +601,16 @@
       </c>
       <c r="G2"/>
       <c r="H2"/>
-      <c r="I2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
         <v>0.0164998065356796</v>
@@ -630,17 +623,16 @@
       </c>
       <c r="G3"/>
       <c r="H3"/>
-      <c r="I3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
         <v>0.00065224547308039</v>
@@ -653,17 +645,16 @@
       </c>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
         <v>0.0840181310144708</v>
@@ -676,17 +667,16 @@
       </c>
       <c r="G5"/>
       <c r="H5"/>
-      <c r="I5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
         <v>0.0160367928499266</v>
@@ -699,17 +689,16 @@
       </c>
       <c r="G6"/>
       <c r="H6"/>
-      <c r="I6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
         <v>0.00983594256126937</v>
@@ -722,17 +711,16 @@
       </c>
       <c r="G7"/>
       <c r="H7"/>
-      <c r="I7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
         <v>-0.102715834816381</v>
@@ -745,17 +733,16 @@
       </c>
       <c r="G8"/>
       <c r="H8"/>
-      <c r="I8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
         <v>0.1052517143198</v>
@@ -768,17 +755,16 @@
       </c>
       <c r="G9"/>
       <c r="H9"/>
-      <c r="I9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
         <v>-0.118090119538363</v>
@@ -791,17 +777,16 @@
       </c>
       <c r="G10"/>
       <c r="H10"/>
-      <c r="I10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
         <v>0.0703905355048749</v>
@@ -814,17 +799,16 @@
       </c>
       <c r="G11"/>
       <c r="H11"/>
-      <c r="I11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
         <v>-0.115775266535295</v>
@@ -837,17 +821,16 @@
       </c>
       <c r="G12"/>
       <c r="H12"/>
-      <c r="I12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
         <v>0.17673132101363</v>
@@ -860,17 +843,16 @@
       </c>
       <c r="G13"/>
       <c r="H13"/>
-      <c r="I13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" t="n">
         <v>0.00620750615759553</v>
@@ -883,17 +865,16 @@
       </c>
       <c r="G14"/>
       <c r="H14"/>
-      <c r="I14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" t="n">
         <v>0.00713761272197522</v>
@@ -906,17 +887,16 @@
       </c>
       <c r="G15"/>
       <c r="H15"/>
-      <c r="I15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" t="n">
         <v>0.0296371350882687</v>
@@ -929,17 +909,16 @@
       </c>
       <c r="G16"/>
       <c r="H16"/>
-      <c r="I16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" t="n">
         <v>-0.036607693468954</v>
@@ -952,17 +931,16 @@
       </c>
       <c r="G17"/>
       <c r="H17"/>
-      <c r="I17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" t="n">
         <v>-0.0168770929595755</v>
@@ -975,17 +953,16 @@
       </c>
       <c r="G18"/>
       <c r="H18"/>
-      <c r="I18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" t="n">
         <v>0.00513284709983518</v>
@@ -998,17 +975,16 @@
       </c>
       <c r="G19"/>
       <c r="H19"/>
-      <c r="I19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" t="n">
         <v>-0.00682196906601559</v>
@@ -1021,17 +997,16 @@
       </c>
       <c r="G20"/>
       <c r="H20"/>
-      <c r="I20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21" t="n">
         <v>0.0382418583576679</v>
@@ -1044,17 +1019,16 @@
       </c>
       <c r="G21"/>
       <c r="H21"/>
-      <c r="I21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22" t="n">
         <v>-0.00735778018481538</v>
@@ -1067,17 +1041,16 @@
       </c>
       <c r="G22"/>
       <c r="H22"/>
-      <c r="I22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" t="n">
         <v>0.0165351194725005</v>
@@ -1090,17 +1063,16 @@
       </c>
       <c r="G23"/>
       <c r="H23"/>
-      <c r="I23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D24" t="n">
         <v>-0.0185968615643766</v>
@@ -1113,17 +1085,16 @@
       </c>
       <c r="G24"/>
       <c r="H24"/>
-      <c r="I24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
         <v>21</v>
-      </c>
-      <c r="B25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" t="s">
-        <v>22</v>
       </c>
       <c r="D25" t="n">
         <v>0.0728360080369906</v>
@@ -1136,17 +1107,16 @@
       </c>
       <c r="G25"/>
       <c r="H25"/>
-      <c r="I25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" t="n">
         <v>-0.0282479596820163</v>
@@ -1159,17 +1129,16 @@
       </c>
       <c r="G26"/>
       <c r="H26"/>
-      <c r="I26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" t="n">
         <v>-0.174783134081328</v>
@@ -1182,17 +1151,16 @@
       </c>
       <c r="G27"/>
       <c r="H27"/>
-      <c r="I27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D28" t="n">
         <v>0.157032962373461</v>
@@ -1205,17 +1173,16 @@
       </c>
       <c r="G28"/>
       <c r="H28"/>
-      <c r="I28"/>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D29" t="n">
         <v>-0.140563115139643</v>
@@ -1228,17 +1195,16 @@
       </c>
       <c r="G29"/>
       <c r="H29"/>
-      <c r="I29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D30" t="n">
         <v>-0.0482262037767428</v>
@@ -1251,17 +1217,16 @@
       </c>
       <c r="G30"/>
       <c r="H30"/>
-      <c r="I30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" t="n">
         <v>0.182486265530603</v>
@@ -1274,17 +1239,16 @@
       </c>
       <c r="G31"/>
       <c r="H31"/>
-      <c r="I31"/>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D32" t="n">
         <v>0.0616244307168021</v>
@@ -1297,17 +1261,16 @@
       </c>
       <c r="G32"/>
       <c r="H32"/>
-      <c r="I32"/>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D33" t="n">
         <v>0.0294183913497299</v>
@@ -1320,17 +1283,16 @@
       </c>
       <c r="G33"/>
       <c r="H33"/>
-      <c r="I33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D34" t="n">
         <v>0.0933746546791991</v>
@@ -1343,17 +1305,16 @@
       </c>
       <c r="G34"/>
       <c r="H34"/>
-      <c r="I34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D35" t="n">
         <v>-0.0859094248008704</v>
@@ -1366,17 +1327,16 @@
       </c>
       <c r="G35"/>
       <c r="H35"/>
-      <c r="I35"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D36" t="n">
         <v>0.0638551652923891</v>
@@ -1389,17 +1349,16 @@
       </c>
       <c r="G36"/>
       <c r="H36"/>
-      <c r="I36"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
         <v>-0.174662039385145</v>
@@ -1412,17 +1371,16 @@
       </c>
       <c r="G37"/>
       <c r="H37"/>
-      <c r="I37"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D38" t="n">
         <v>0.130769293679604</v>
@@ -1435,17 +1393,16 @@
       </c>
       <c r="G38"/>
       <c r="H38"/>
-      <c r="I38"/>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D39" t="n">
         <v>-0.101639507795085</v>
@@ -1458,17 +1415,16 @@
       </c>
       <c r="G39"/>
       <c r="H39"/>
-      <c r="I39"/>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D40" t="n">
         <v>0.12027851759581</v>
@@ -1481,17 +1437,16 @@
       </c>
       <c r="G40"/>
       <c r="H40"/>
-      <c r="I40"/>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" t="n">
         <v>0.0405545434450909</v>
@@ -1504,17 +1459,16 @@
       </c>
       <c r="G41"/>
       <c r="H41"/>
-      <c r="I41"/>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D42" t="n">
         <v>0.0023391557339578</v>
@@ -1527,17 +1481,16 @@
       </c>
       <c r="G42"/>
       <c r="H42"/>
-      <c r="I42"/>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D43" t="n">
         <v>0.0525217862080328</v>
@@ -1550,17 +1503,16 @@
       </c>
       <c r="G43"/>
       <c r="H43"/>
-      <c r="I43"/>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D44" t="n">
         <v>0.04523826678797</v>
@@ -1573,17 +1525,16 @@
       </c>
       <c r="G44"/>
       <c r="H44"/>
-      <c r="I44"/>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D45" t="n">
         <v>0.0430142920971172</v>
@@ -1596,17 +1547,16 @@
       </c>
       <c r="G45"/>
       <c r="H45"/>
-      <c r="I45"/>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" t="n">
         <v>-0.0870395789449637</v>
@@ -1619,17 +1569,16 @@
       </c>
       <c r="G46"/>
       <c r="H46"/>
-      <c r="I46"/>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D47" t="n">
         <v>-0.030434410883923</v>
@@ -1642,17 +1591,16 @@
       </c>
       <c r="G47"/>
       <c r="H47"/>
-      <c r="I47"/>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" t="n">
         <v>-0.0525746278049512</v>
@@ -1665,17 +1613,16 @@
       </c>
       <c r="G48"/>
       <c r="H48"/>
-      <c r="I48"/>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D49" t="n">
         <v>-0.0223069136055875</v>
@@ -1688,17 +1635,16 @@
       </c>
       <c r="G49"/>
       <c r="H49"/>
-      <c r="I49"/>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D50" t="n">
         <v>-0.0148843622656003</v>
@@ -1711,17 +1657,16 @@
       </c>
       <c r="G50"/>
       <c r="H50"/>
-      <c r="I50"/>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D51" t="n">
         <v>-0.0518772222493833</v>
@@ -1734,17 +1679,16 @@
       </c>
       <c r="G51"/>
       <c r="H51"/>
-      <c r="I51"/>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D52" t="n">
         <v>0.0453289188205259</v>
@@ -1757,17 +1701,16 @@
       </c>
       <c r="G52"/>
       <c r="H52"/>
-      <c r="I52"/>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C53" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D53" t="n">
         <v>0.00468438006438979</v>
@@ -1780,17 +1723,16 @@
       </c>
       <c r="G53"/>
       <c r="H53"/>
-      <c r="I53"/>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D54" t="n">
         <v>0.0506275924890334</v>
@@ -1803,17 +1745,16 @@
       </c>
       <c r="G54"/>
       <c r="H54"/>
-      <c r="I54"/>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D55" t="n">
         <v>0.00484475146308899</v>
@@ -1826,17 +1767,16 @@
       </c>
       <c r="G55"/>
       <c r="H55"/>
-      <c r="I55"/>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C56" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D56" t="n">
         <v>0.0573564263286989</v>
@@ -1849,17 +1789,16 @@
       </c>
       <c r="G56"/>
       <c r="H56"/>
-      <c r="I56"/>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C57" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D57" t="n">
         <v>-0.0306300639225915</v>
@@ -1872,17 +1811,16 @@
       </c>
       <c r="G57"/>
       <c r="H57"/>
-      <c r="I57"/>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D58" t="n">
         <v>0.0591895800604847</v>
@@ -1895,17 +1833,16 @@
       </c>
       <c r="G58"/>
       <c r="H58"/>
-      <c r="I58"/>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C59" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D59" t="n">
         <v>-0.0881528900574695</v>
@@ -1918,17 +1855,16 @@
       </c>
       <c r="G59"/>
       <c r="H59"/>
-      <c r="I59"/>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C60" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D60" t="n">
         <v>0.0325143262666986</v>
@@ -1941,17 +1877,16 @@
       </c>
       <c r="G60"/>
       <c r="H60"/>
-      <c r="I60"/>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D61" t="n">
         <v>-0.0954318394594336</v>
@@ -1964,17 +1899,16 @@
       </c>
       <c r="G61"/>
       <c r="H61"/>
-      <c r="I61"/>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D62" t="n">
         <v>0.0855872427333253</v>
@@ -1987,17 +1921,16 @@
       </c>
       <c r="G62"/>
       <c r="H62"/>
-      <c r="I62"/>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D63" t="n">
         <v>-0.042515028435679</v>
@@ -2010,17 +1943,16 @@
       </c>
       <c r="G63"/>
       <c r="H63"/>
-      <c r="I63"/>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D64" t="n">
         <v>0.0163440292053376</v>
@@ -2033,17 +1965,16 @@
       </c>
       <c r="G64"/>
       <c r="H64"/>
-      <c r="I64"/>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C65" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D65" t="n">
         <v>0.125310204547815</v>
@@ -2056,17 +1987,16 @@
       </c>
       <c r="G65"/>
       <c r="H65"/>
-      <c r="I65"/>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D66" t="n">
         <v>0.0835414782985354</v>
@@ -2079,17 +2009,16 @@
       </c>
       <c r="G66"/>
       <c r="H66"/>
-      <c r="I66"/>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C67" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D67" t="n">
         <v>0.00954784692452318</v>
@@ -2102,17 +2031,16 @@
       </c>
       <c r="G67"/>
       <c r="H67"/>
-      <c r="I67"/>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C68" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D68" t="n">
         <v>-0.0385374394216661</v>
@@ -2125,17 +2053,16 @@
       </c>
       <c r="G68"/>
       <c r="H68"/>
-      <c r="I68"/>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D69" t="n">
         <v>0.0363797920395403</v>
@@ -2148,17 +2075,16 @@
       </c>
       <c r="G69"/>
       <c r="H69"/>
-      <c r="I69"/>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C70" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D70" t="n">
         <v>-0.0515427592930625</v>
@@ -2171,17 +2097,16 @@
       </c>
       <c r="G70"/>
       <c r="H70"/>
-      <c r="I70"/>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C71" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D71" t="n">
         <v>-0.0342974740250952</v>
@@ -2194,17 +2119,16 @@
       </c>
       <c r="G71"/>
       <c r="H71"/>
-      <c r="I71"/>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B72" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D72" t="n">
         <v>-0.0646640787042194</v>
@@ -2217,17 +2141,16 @@
       </c>
       <c r="G72"/>
       <c r="H72"/>
-      <c r="I72"/>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C73" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D73" t="n">
         <v>0.00846347351720542</v>
@@ -2240,17 +2163,16 @@
       </c>
       <c r="G73"/>
       <c r="H73"/>
-      <c r="I73"/>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D74" t="n">
         <v>-0.0734300106282945</v>
@@ -2263,17 +2185,16 @@
       </c>
       <c r="G74"/>
       <c r="H74"/>
-      <c r="I74"/>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D75" t="n">
         <v>-0.115658654721923</v>
@@ -2286,17 +2207,16 @@
       </c>
       <c r="G75"/>
       <c r="H75"/>
-      <c r="I75"/>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C76" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D76" t="n">
         <v>0.0530984739829882</v>
@@ -2309,17 +2229,16 @@
       </c>
       <c r="G76"/>
       <c r="H76"/>
-      <c r="I76"/>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D77" t="n">
         <v>-0.055807454036919</v>
@@ -2332,17 +2251,16 @@
       </c>
       <c r="G77"/>
       <c r="H77"/>
-      <c r="I77"/>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D78" t="n">
         <v>0.0329761187878349</v>
@@ -2355,17 +2273,16 @@
       </c>
       <c r="G78"/>
       <c r="H78"/>
-      <c r="I78"/>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D79" t="n">
         <v>0.139512326247094</v>
@@ -2378,17 +2295,16 @@
       </c>
       <c r="G79"/>
       <c r="H79"/>
-      <c r="I79"/>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C80" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D80" t="n">
         <v>-0.022151275492834</v>
@@ -2401,17 +2317,16 @@
       </c>
       <c r="G80"/>
       <c r="H80"/>
-      <c r="I80"/>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D81" t="n">
         <v>0.022783891292153</v>
@@ -2424,17 +2339,16 @@
       </c>
       <c r="G81"/>
       <c r="H81"/>
-      <c r="I81"/>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C82" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D82" t="n">
         <v>0.1288714743311</v>
@@ -2447,17 +2361,16 @@
       </c>
       <c r="G82"/>
       <c r="H82"/>
-      <c r="I82"/>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D83" t="n">
         <v>-0.0897724879420425</v>
@@ -2470,17 +2383,16 @@
       </c>
       <c r="G83"/>
       <c r="H83"/>
-      <c r="I83"/>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C84" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D84" t="n">
         <v>0.0517657143931209</v>
@@ -2493,17 +2405,16 @@
       </c>
       <c r="G84"/>
       <c r="H84"/>
-      <c r="I84"/>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C85" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D85" t="n">
         <v>-0.143891652262352</v>
@@ -2516,17 +2427,16 @@
       </c>
       <c r="G85"/>
       <c r="H85"/>
-      <c r="I85"/>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B86" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D86" t="n">
         <v>0.100471604998926</v>
@@ -2539,17 +2449,16 @@
       </c>
       <c r="G86"/>
       <c r="H86"/>
-      <c r="I86"/>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C87" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D87" t="n">
         <v>0.00936219381370434</v>
@@ -2562,17 +2471,16 @@
       </c>
       <c r="G87"/>
       <c r="H87"/>
-      <c r="I87"/>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C88" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D88" t="n">
         <v>-0.0289848896151883</v>
@@ -2585,17 +2493,16 @@
       </c>
       <c r="G88"/>
       <c r="H88"/>
-      <c r="I88"/>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C89" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D89" t="n">
         <v>0.120625824483425</v>
@@ -2608,17 +2515,16 @@
       </c>
       <c r="G89"/>
       <c r="H89"/>
-      <c r="I89"/>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D90" t="n">
         <v>0.0329138858095021</v>
@@ -2631,17 +2537,16 @@
       </c>
       <c r="G90"/>
       <c r="H90"/>
-      <c r="I90"/>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C91" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D91" t="n">
         <v>0.00470309546143418</v>
@@ -2654,17 +2559,16 @@
       </c>
       <c r="G91"/>
       <c r="H91"/>
-      <c r="I91"/>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B92" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D92" t="n">
         <v>-0.095893865750365</v>
@@ -2677,17 +2581,16 @@
       </c>
       <c r="G92"/>
       <c r="H92"/>
-      <c r="I92"/>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B93" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C93" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D93" t="n">
         <v>0.0670098559621318</v>
@@ -2700,17 +2603,16 @@
       </c>
       <c r="G93"/>
       <c r="H93"/>
-      <c r="I93"/>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C94" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D94" t="n">
         <v>-0.110732339353547</v>
@@ -2723,17 +2625,16 @@
       </c>
       <c r="G94"/>
       <c r="H94"/>
-      <c r="I94"/>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B95" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C95" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D95" t="n">
         <v>0.0538554160323744</v>
@@ -2746,17 +2647,16 @@
       </c>
       <c r="G95"/>
       <c r="H95"/>
-      <c r="I95"/>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B96" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C96" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D96" t="n">
         <v>-0.097178404970918</v>
@@ -2769,17 +2669,16 @@
       </c>
       <c r="G96"/>
       <c r="H96"/>
-      <c r="I96"/>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B97" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C97" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
         <v>0.103895312976639</v>
@@ -2792,17 +2691,16 @@
       </c>
       <c r="G97"/>
       <c r="H97"/>
-      <c r="I97"/>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B98" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C98" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D98" t="n">
         <v>-0.15901725336162</v>
@@ -2815,17 +2713,16 @@
       </c>
       <c r="G98"/>
       <c r="H98"/>
-      <c r="I98"/>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C99" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D99" t="n">
         <v>-0.0731436262862439</v>
@@ -2838,17 +2735,16 @@
       </c>
       <c r="G99"/>
       <c r="H99"/>
-      <c r="I99"/>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C100" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D100" t="n">
         <v>0.0367544447776506</v>
@@ -2861,17 +2757,16 @@
       </c>
       <c r="G100"/>
       <c r="H100"/>
-      <c r="I100"/>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C101" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D101" t="n">
         <v>-0.181117658584734</v>
@@ -2884,17 +2779,16 @@
       </c>
       <c r="G101"/>
       <c r="H101"/>
-      <c r="I101"/>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D102" t="n">
         <v>-0.0505653595107006</v>
@@ -2907,17 +2801,16 @@
       </c>
       <c r="G102"/>
       <c r="H102"/>
-      <c r="I102"/>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C103" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D103" t="n">
         <v>0.12996447932257</v>
@@ -2930,17 +2823,16 @@
       </c>
       <c r="G103"/>
       <c r="H103"/>
-      <c r="I103"/>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C104" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D104" t="n">
         <v>0.0163861639288321</v>
@@ -2953,17 +2845,16 @@
       </c>
       <c r="G104"/>
       <c r="H104"/>
-      <c r="I104"/>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C105" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D105" t="n">
         <v>-0.0135959007473873</v>
@@ -2976,17 +2867,16 @@
       </c>
       <c r="G105"/>
       <c r="H105"/>
-      <c r="I105"/>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B106" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C106" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D106" t="n">
         <v>0.180414233624163</v>
@@ -2999,17 +2889,16 @@
       </c>
       <c r="G106"/>
       <c r="H106"/>
-      <c r="I106"/>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B107" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C107" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D107" t="n">
         <v>-0.0554750139169474</v>
@@ -3022,17 +2911,16 @@
       </c>
       <c r="G107"/>
       <c r="H107"/>
-      <c r="I107"/>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C108" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D108" t="n">
         <v>0.11642979309734</v>
@@ -3045,17 +2933,16 @@
       </c>
       <c r="G108"/>
       <c r="H108"/>
-      <c r="I108"/>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B109" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C109" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D109" t="n">
         <v>-0.152355125779557</v>
@@ -3068,7 +2955,6 @@
       </c>
       <c r="G109"/>
       <c r="H109"/>
-      <c r="I109"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3086,19 +2972,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>32</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>33</v>
-      </c>
-      <c r="F1" t="s">
-        <v>34</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -3107,21 +2993,21 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" t="s">
         <v>35</v>
-      </c>
-      <c r="J1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
         <v>37</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -3138,18 +3024,18 @@
         <v>359</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
         <v>40</v>
-      </c>
-      <c r="C3" t="s">
-        <v>41</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -3166,18 +3052,18 @@
         <v>174</v>
       </c>
       <c r="J3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
         <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>44</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -3194,18 +3080,18 @@
         <v>164</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
         <v>46</v>
-      </c>
-      <c r="C5" t="s">
-        <v>47</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -3222,18 +3108,18 @@
         <v>159</v>
       </c>
       <c r="J5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -3250,18 +3136,18 @@
         <v>156</v>
       </c>
       <c r="J6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -3278,18 +3164,18 @@
         <v>143</v>
       </c>
       <c r="J7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -3306,18 +3192,18 @@
         <v>134</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
         <v>55</v>
-      </c>
-      <c r="C9" t="s">
-        <v>56</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -3334,18 +3220,18 @@
         <v>81</v>
       </c>
       <c r="J9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
         <v>58</v>
-      </c>
-      <c r="C10" t="s">
-        <v>59</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
@@ -3362,18 +3248,18 @@
         <v>76</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -3390,18 +3276,18 @@
         <v>68</v>
       </c>
       <c r="J11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
         <v>63</v>
-      </c>
-      <c r="C12" t="s">
-        <v>64</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -3418,18 +3304,18 @@
         <v>63</v>
       </c>
       <c r="J12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" t="s">
         <v>66</v>
-      </c>
-      <c r="C13" t="s">
-        <v>67</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -3446,7 +3332,7 @@
         <v>58</v>
       </c>
       <c r="J13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3485,19 +3371,16 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>0.106679111156521</v>
@@ -3510,17 +3393,16 @@
       </c>
       <c r="G2"/>
       <c r="H2"/>
-      <c r="I2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
         <v>0.0164998065356796</v>
@@ -3533,17 +3415,16 @@
       </c>
       <c r="G3"/>
       <c r="H3"/>
-      <c r="I3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
         <v>0.00065224547308039</v>
@@ -3556,17 +3437,16 @@
       </c>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
         <v>0.0840181310144708</v>
@@ -3579,17 +3459,16 @@
       </c>
       <c r="G5"/>
       <c r="H5"/>
-      <c r="I5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
         <v>0.0160367928499266</v>
@@ -3602,17 +3481,16 @@
       </c>
       <c r="G6"/>
       <c r="H6"/>
-      <c r="I6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
         <v>0.00983594256126937</v>
@@ -3625,17 +3503,16 @@
       </c>
       <c r="G7"/>
       <c r="H7"/>
-      <c r="I7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
         <v>-0.102715834816381</v>
@@ -3648,17 +3525,16 @@
       </c>
       <c r="G8"/>
       <c r="H8"/>
-      <c r="I8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
         <v>0.1052517143198</v>
@@ -3671,17 +3547,16 @@
       </c>
       <c r="G9"/>
       <c r="H9"/>
-      <c r="I9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
         <v>-0.118090119538363</v>
@@ -3694,17 +3569,16 @@
       </c>
       <c r="G10"/>
       <c r="H10"/>
-      <c r="I10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
         <v>0.0703905355048749</v>
@@ -3717,17 +3591,16 @@
       </c>
       <c r="G11"/>
       <c r="H11"/>
-      <c r="I11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
         <v>-0.115775266535295</v>
@@ -3740,17 +3613,16 @@
       </c>
       <c r="G12"/>
       <c r="H12"/>
-      <c r="I12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
         <v>0.17673132101363</v>
@@ -3763,17 +3635,16 @@
       </c>
       <c r="G13"/>
       <c r="H13"/>
-      <c r="I13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" t="n">
         <v>0.00620750615759553</v>
@@ -3786,17 +3657,16 @@
       </c>
       <c r="G14"/>
       <c r="H14"/>
-      <c r="I14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" t="n">
         <v>0.00713761272197522</v>
@@ -3809,17 +3679,16 @@
       </c>
       <c r="G15"/>
       <c r="H15"/>
-      <c r="I15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" t="n">
         <v>0.0296371350882687</v>
@@ -3832,17 +3701,16 @@
       </c>
       <c r="G16"/>
       <c r="H16"/>
-      <c r="I16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" t="n">
         <v>-0.036607693468954</v>
@@ -3855,17 +3723,16 @@
       </c>
       <c r="G17"/>
       <c r="H17"/>
-      <c r="I17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" t="n">
         <v>-0.0168770929595755</v>
@@ -3878,17 +3745,16 @@
       </c>
       <c r="G18"/>
       <c r="H18"/>
-      <c r="I18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" t="n">
         <v>0.00513284709983518</v>
@@ -3901,17 +3767,16 @@
       </c>
       <c r="G19"/>
       <c r="H19"/>
-      <c r="I19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20" t="n">
         <v>-0.00682196906601559</v>
@@ -3924,17 +3789,16 @@
       </c>
       <c r="G20"/>
       <c r="H20"/>
-      <c r="I20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21" t="n">
         <v>0.0382418583576679</v>
@@ -3947,17 +3811,16 @@
       </c>
       <c r="G21"/>
       <c r="H21"/>
-      <c r="I21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22" t="n">
         <v>-0.00735778018481538</v>
@@ -3970,17 +3833,16 @@
       </c>
       <c r="G22"/>
       <c r="H22"/>
-      <c r="I22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" t="n">
         <v>0.0165351194725005</v>
@@ -3993,17 +3855,16 @@
       </c>
       <c r="G23"/>
       <c r="H23"/>
-      <c r="I23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D24" t="n">
         <v>-0.0185968615643766</v>
@@ -4016,17 +3877,16 @@
       </c>
       <c r="G24"/>
       <c r="H24"/>
-      <c r="I24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
         <v>21</v>
-      </c>
-      <c r="B25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" t="s">
-        <v>22</v>
       </c>
       <c r="D25" t="n">
         <v>0.0728360080369906</v>
@@ -4039,17 +3899,16 @@
       </c>
       <c r="G25"/>
       <c r="H25"/>
-      <c r="I25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D26" t="n">
         <v>-0.0282479596820163</v>
@@ -4062,17 +3921,16 @@
       </c>
       <c r="G26"/>
       <c r="H26"/>
-      <c r="I26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" t="n">
         <v>-0.174783134081328</v>
@@ -4085,17 +3943,16 @@
       </c>
       <c r="G27"/>
       <c r="H27"/>
-      <c r="I27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D28" t="n">
         <v>0.157032962373461</v>
@@ -4108,17 +3965,16 @@
       </c>
       <c r="G28"/>
       <c r="H28"/>
-      <c r="I28"/>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D29" t="n">
         <v>-0.140563115139643</v>
@@ -4131,17 +3987,16 @@
       </c>
       <c r="G29"/>
       <c r="H29"/>
-      <c r="I29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D30" t="n">
         <v>-0.0482262037767428</v>
@@ -4154,17 +4009,16 @@
       </c>
       <c r="G30"/>
       <c r="H30"/>
-      <c r="I30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" t="n">
         <v>0.182486265530603</v>
@@ -4177,17 +4031,16 @@
       </c>
       <c r="G31"/>
       <c r="H31"/>
-      <c r="I31"/>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D32" t="n">
         <v>0.0616244307168021</v>
@@ -4200,17 +4053,16 @@
       </c>
       <c r="G32"/>
       <c r="H32"/>
-      <c r="I32"/>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C33" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D33" t="n">
         <v>0.0294183913497299</v>
@@ -4223,17 +4075,16 @@
       </c>
       <c r="G33"/>
       <c r="H33"/>
-      <c r="I33"/>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D34" t="n">
         <v>0.0933746546791991</v>
@@ -4246,17 +4097,16 @@
       </c>
       <c r="G34"/>
       <c r="H34"/>
-      <c r="I34"/>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D35" t="n">
         <v>-0.0859094248008704</v>
@@ -4269,17 +4119,16 @@
       </c>
       <c r="G35"/>
       <c r="H35"/>
-      <c r="I35"/>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D36" t="n">
         <v>0.0638551652923891</v>
@@ -4292,17 +4141,16 @@
       </c>
       <c r="G36"/>
       <c r="H36"/>
-      <c r="I36"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
         <v>-0.174662039385145</v>
@@ -4315,17 +4163,16 @@
       </c>
       <c r="G37"/>
       <c r="H37"/>
-      <c r="I37"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D38" t="n">
         <v>0.130769293679604</v>
@@ -4338,17 +4185,16 @@
       </c>
       <c r="G38"/>
       <c r="H38"/>
-      <c r="I38"/>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D39" t="n">
         <v>-0.101639507795085</v>
@@ -4361,17 +4207,16 @@
       </c>
       <c r="G39"/>
       <c r="H39"/>
-      <c r="I39"/>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D40" t="n">
         <v>0.12027851759581</v>
@@ -4384,17 +4229,16 @@
       </c>
       <c r="G40"/>
       <c r="H40"/>
-      <c r="I40"/>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" t="n">
         <v>0.0405545434450909</v>
@@ -4407,17 +4251,16 @@
       </c>
       <c r="G41"/>
       <c r="H41"/>
-      <c r="I41"/>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D42" t="n">
         <v>0.0023391557339578</v>
@@ -4430,17 +4273,16 @@
       </c>
       <c r="G42"/>
       <c r="H42"/>
-      <c r="I42"/>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D43" t="n">
         <v>0.0525217862080328</v>
@@ -4453,17 +4295,16 @@
       </c>
       <c r="G43"/>
       <c r="H43"/>
-      <c r="I43"/>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D44" t="n">
         <v>0.04523826678797</v>
@@ -4476,17 +4317,16 @@
       </c>
       <c r="G44"/>
       <c r="H44"/>
-      <c r="I44"/>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D45" t="n">
         <v>0.0430142920971172</v>
@@ -4499,17 +4339,16 @@
       </c>
       <c r="G45"/>
       <c r="H45"/>
-      <c r="I45"/>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" t="n">
         <v>-0.0870395789449637</v>
@@ -4522,17 +4361,16 @@
       </c>
       <c r="G46"/>
       <c r="H46"/>
-      <c r="I46"/>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D47" t="n">
         <v>-0.030434410883923</v>
@@ -4545,17 +4383,16 @@
       </c>
       <c r="G47"/>
       <c r="H47"/>
-      <c r="I47"/>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B48" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" t="n">
         <v>-0.0525746278049512</v>
@@ -4568,17 +4405,16 @@
       </c>
       <c r="G48"/>
       <c r="H48"/>
-      <c r="I48"/>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D49" t="n">
         <v>-0.0223069136055875</v>
@@ -4591,17 +4427,16 @@
       </c>
       <c r="G49"/>
       <c r="H49"/>
-      <c r="I49"/>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D50" t="n">
         <v>-0.0148843622656003</v>
@@ -4614,17 +4449,16 @@
       </c>
       <c r="G50"/>
       <c r="H50"/>
-      <c r="I50"/>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D51" t="n">
         <v>-0.0518772222493833</v>
@@ -4637,17 +4471,16 @@
       </c>
       <c r="G51"/>
       <c r="H51"/>
-      <c r="I51"/>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C52" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D52" t="n">
         <v>0.0453289188205259</v>
@@ -4660,17 +4493,16 @@
       </c>
       <c r="G52"/>
       <c r="H52"/>
-      <c r="I52"/>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C53" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D53" t="n">
         <v>0.00468438006438979</v>
@@ -4683,17 +4515,16 @@
       </c>
       <c r="G53"/>
       <c r="H53"/>
-      <c r="I53"/>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B54" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D54" t="n">
         <v>0.0506275924890334</v>
@@ -4706,17 +4537,16 @@
       </c>
       <c r="G54"/>
       <c r="H54"/>
-      <c r="I54"/>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D55" t="n">
         <v>0.00484475146308899</v>
@@ -4729,17 +4559,16 @@
       </c>
       <c r="G55"/>
       <c r="H55"/>
-      <c r="I55"/>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C56" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D56" t="n">
         <v>0.0573564263286989</v>
@@ -4752,17 +4581,16 @@
       </c>
       <c r="G56"/>
       <c r="H56"/>
-      <c r="I56"/>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C57" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D57" t="n">
         <v>-0.0306300639225915</v>
@@ -4775,17 +4603,16 @@
       </c>
       <c r="G57"/>
       <c r="H57"/>
-      <c r="I57"/>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D58" t="n">
         <v>0.0591895800604847</v>
@@ -4798,17 +4625,16 @@
       </c>
       <c r="G58"/>
       <c r="H58"/>
-      <c r="I58"/>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C59" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D59" t="n">
         <v>-0.0881528900574695</v>
@@ -4821,17 +4647,16 @@
       </c>
       <c r="G59"/>
       <c r="H59"/>
-      <c r="I59"/>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B60" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C60" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D60" t="n">
         <v>0.0325143262666986</v>
@@ -4844,17 +4669,16 @@
       </c>
       <c r="G60"/>
       <c r="H60"/>
-      <c r="I60"/>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D61" t="n">
         <v>-0.0954318394594336</v>
@@ -4867,17 +4691,16 @@
       </c>
       <c r="G61"/>
       <c r="H61"/>
-      <c r="I61"/>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D62" t="n">
         <v>0.0855872427333253</v>
@@ -4890,17 +4713,16 @@
       </c>
       <c r="G62"/>
       <c r="H62"/>
-      <c r="I62"/>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B63" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C63" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D63" t="n">
         <v>-0.042515028435679</v>
@@ -4913,17 +4735,16 @@
       </c>
       <c r="G63"/>
       <c r="H63"/>
-      <c r="I63"/>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C64" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D64" t="n">
         <v>0.0163440292053376</v>
@@ -4936,17 +4757,16 @@
       </c>
       <c r="G64"/>
       <c r="H64"/>
-      <c r="I64"/>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C65" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D65" t="n">
         <v>0.125310204547815</v>
@@ -4959,17 +4779,16 @@
       </c>
       <c r="G65"/>
       <c r="H65"/>
-      <c r="I65"/>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D66" t="n">
         <v>0.0835414782985354</v>
@@ -4982,17 +4801,16 @@
       </c>
       <c r="G66"/>
       <c r="H66"/>
-      <c r="I66"/>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C67" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D67" t="n">
         <v>0.00954784692452318</v>
@@ -5005,17 +4823,16 @@
       </c>
       <c r="G67"/>
       <c r="H67"/>
-      <c r="I67"/>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C68" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D68" t="n">
         <v>-0.0385374394216661</v>
@@ -5028,17 +4845,16 @@
       </c>
       <c r="G68"/>
       <c r="H68"/>
-      <c r="I68"/>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C69" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D69" t="n">
         <v>0.0363797920395403</v>
@@ -5051,17 +4867,16 @@
       </c>
       <c r="G69"/>
       <c r="H69"/>
-      <c r="I69"/>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C70" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D70" t="n">
         <v>-0.0515427592930625</v>
@@ -5074,17 +4889,16 @@
       </c>
       <c r="G70"/>
       <c r="H70"/>
-      <c r="I70"/>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C71" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D71" t="n">
         <v>-0.0342974740250952</v>
@@ -5097,17 +4911,16 @@
       </c>
       <c r="G71"/>
       <c r="H71"/>
-      <c r="I71"/>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B72" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D72" t="n">
         <v>-0.0646640787042194</v>
@@ -5120,17 +4933,16 @@
       </c>
       <c r="G72"/>
       <c r="H72"/>
-      <c r="I72"/>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C73" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D73" t="n">
         <v>0.00846347351720542</v>
@@ -5143,17 +4955,16 @@
       </c>
       <c r="G73"/>
       <c r="H73"/>
-      <c r="I73"/>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C74" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D74" t="n">
         <v>-0.0734300106282945</v>
@@ -5166,17 +4977,16 @@
       </c>
       <c r="G74"/>
       <c r="H74"/>
-      <c r="I74"/>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D75" t="n">
         <v>-0.115658654721923</v>
@@ -5189,17 +4999,16 @@
       </c>
       <c r="G75"/>
       <c r="H75"/>
-      <c r="I75"/>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C76" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D76" t="n">
         <v>0.0530984739829882</v>
@@ -5212,17 +5021,16 @@
       </c>
       <c r="G76"/>
       <c r="H76"/>
-      <c r="I76"/>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C77" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D77" t="n">
         <v>-0.055807454036919</v>
@@ -5235,17 +5043,16 @@
       </c>
       <c r="G77"/>
       <c r="H77"/>
-      <c r="I77"/>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D78" t="n">
         <v>0.0329761187878349</v>
@@ -5258,17 +5065,16 @@
       </c>
       <c r="G78"/>
       <c r="H78"/>
-      <c r="I78"/>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B79" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C79" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D79" t="n">
         <v>0.139512326247094</v>
@@ -5281,17 +5087,16 @@
       </c>
       <c r="G79"/>
       <c r="H79"/>
-      <c r="I79"/>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C80" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D80" t="n">
         <v>-0.022151275492834</v>
@@ -5304,17 +5109,16 @@
       </c>
       <c r="G80"/>
       <c r="H80"/>
-      <c r="I80"/>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D81" t="n">
         <v>0.022783891292153</v>
@@ -5327,17 +5131,16 @@
       </c>
       <c r="G81"/>
       <c r="H81"/>
-      <c r="I81"/>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C82" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D82" t="n">
         <v>0.1288714743311</v>
@@ -5350,17 +5153,16 @@
       </c>
       <c r="G82"/>
       <c r="H82"/>
-      <c r="I82"/>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D83" t="n">
         <v>-0.0897724879420425</v>
@@ -5373,17 +5175,16 @@
       </c>
       <c r="G83"/>
       <c r="H83"/>
-      <c r="I83"/>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B84" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C84" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D84" t="n">
         <v>0.0517657143931209</v>
@@ -5396,17 +5197,16 @@
       </c>
       <c r="G84"/>
       <c r="H84"/>
-      <c r="I84"/>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B85" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C85" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D85" t="n">
         <v>-0.143891652262352</v>
@@ -5419,17 +5219,16 @@
       </c>
       <c r="G85"/>
       <c r="H85"/>
-      <c r="I85"/>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B86" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D86" t="n">
         <v>0.100471604998926</v>
@@ -5442,17 +5241,16 @@
       </c>
       <c r="G86"/>
       <c r="H86"/>
-      <c r="I86"/>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C87" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D87" t="n">
         <v>0.00936219381370434</v>
@@ -5465,17 +5263,16 @@
       </c>
       <c r="G87"/>
       <c r="H87"/>
-      <c r="I87"/>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B88" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C88" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D88" t="n">
         <v>-0.0289848896151883</v>
@@ -5488,17 +5285,16 @@
       </c>
       <c r="G88"/>
       <c r="H88"/>
-      <c r="I88"/>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B89" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C89" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D89" t="n">
         <v>0.120625824483425</v>
@@ -5511,17 +5307,16 @@
       </c>
       <c r="G89"/>
       <c r="H89"/>
-      <c r="I89"/>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D90" t="n">
         <v>0.0329138858095021</v>
@@ -5534,17 +5329,16 @@
       </c>
       <c r="G90"/>
       <c r="H90"/>
-      <c r="I90"/>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B91" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C91" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D91" t="n">
         <v>0.00470309546143418</v>
@@ -5557,17 +5351,16 @@
       </c>
       <c r="G91"/>
       <c r="H91"/>
-      <c r="I91"/>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B92" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C92" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D92" t="n">
         <v>-0.095893865750365</v>
@@ -5580,17 +5373,16 @@
       </c>
       <c r="G92"/>
       <c r="H92"/>
-      <c r="I92"/>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B93" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C93" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D93" t="n">
         <v>0.0670098559621318</v>
@@ -5603,17 +5395,16 @@
       </c>
       <c r="G93"/>
       <c r="H93"/>
-      <c r="I93"/>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C94" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D94" t="n">
         <v>-0.110732339353547</v>
@@ -5626,17 +5417,16 @@
       </c>
       <c r="G94"/>
       <c r="H94"/>
-      <c r="I94"/>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B95" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C95" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D95" t="n">
         <v>0.0538554160323744</v>
@@ -5649,17 +5439,16 @@
       </c>
       <c r="G95"/>
       <c r="H95"/>
-      <c r="I95"/>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B96" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C96" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D96" t="n">
         <v>-0.097178404970918</v>
@@ -5672,17 +5461,16 @@
       </c>
       <c r="G96"/>
       <c r="H96"/>
-      <c r="I96"/>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B97" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C97" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
         <v>0.103895312976639</v>
@@ -5695,17 +5483,16 @@
       </c>
       <c r="G97"/>
       <c r="H97"/>
-      <c r="I97"/>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B98" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C98" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D98" t="n">
         <v>-0.15901725336162</v>
@@ -5718,17 +5505,16 @@
       </c>
       <c r="G98"/>
       <c r="H98"/>
-      <c r="I98"/>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B99" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C99" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D99" t="n">
         <v>-0.0731436262862439</v>
@@ -5741,17 +5527,16 @@
       </c>
       <c r="G99"/>
       <c r="H99"/>
-      <c r="I99"/>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B100" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C100" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D100" t="n">
         <v>0.0367544447776506</v>
@@ -5764,17 +5549,16 @@
       </c>
       <c r="G100"/>
       <c r="H100"/>
-      <c r="I100"/>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B101" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C101" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D101" t="n">
         <v>-0.181117658584734</v>
@@ -5787,17 +5571,16 @@
       </c>
       <c r="G101"/>
       <c r="H101"/>
-      <c r="I101"/>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D102" t="n">
         <v>-0.0505653595107006</v>
@@ -5810,17 +5593,16 @@
       </c>
       <c r="G102"/>
       <c r="H102"/>
-      <c r="I102"/>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C103" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D103" t="n">
         <v>0.12996447932257</v>
@@ -5833,17 +5615,16 @@
       </c>
       <c r="G103"/>
       <c r="H103"/>
-      <c r="I103"/>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C104" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D104" t="n">
         <v>0.0163861639288321</v>
@@ -5856,17 +5637,16 @@
       </c>
       <c r="G104"/>
       <c r="H104"/>
-      <c r="I104"/>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B105" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C105" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D105" t="n">
         <v>-0.0135959007473873</v>
@@ -5879,17 +5659,16 @@
       </c>
       <c r="G105"/>
       <c r="H105"/>
-      <c r="I105"/>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B106" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C106" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D106" t="n">
         <v>0.180414233624163</v>
@@ -5902,17 +5681,16 @@
       </c>
       <c r="G106"/>
       <c r="H106"/>
-      <c r="I106"/>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B107" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C107" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D107" t="n">
         <v>-0.0554750139169474</v>
@@ -5925,17 +5703,16 @@
       </c>
       <c r="G107"/>
       <c r="H107"/>
-      <c r="I107"/>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B108" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C108" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D108" t="n">
         <v>0.11642979309734</v>
@@ -5948,17 +5725,16 @@
       </c>
       <c r="G108"/>
       <c r="H108"/>
-      <c r="I108"/>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B109" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C109" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D109" t="n">
         <v>-0.152355125779557</v>
@@ -5971,7 +5747,6 @@
       </c>
       <c r="G109"/>
       <c r="H109"/>
-      <c r="I109"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>